<commit_message>
fix(UI & backend):upcoming test upload problem and practice hindi to english problem fixed
</commit_message>
<xml_diff>
--- a/assets/downloads/weekly_test_upload_template.xlsx
+++ b/assets/downloads/weekly_test_upload_template.xlsx
@@ -8,11 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Questions'!$A$1:$J$1</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -34,10 +32,9 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="000B2F63"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -46,12 +43,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000B2F63"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F4C542"/>
+        <fgColor rgb="000B2D57"/>
       </patternFill>
     </fill>
   </fills>
@@ -67,19 +59,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -445,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -454,10 +442,10 @@
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -512,8 +500,125 @@
         </is>
       </c>
     </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>मैं रोज अंग्रेजी बोलता हूँ।</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>I speak English every day. || I speak English daily.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>hindi_to_english</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Present Simple</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Beginner</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3" ht="42" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Correct: She go to class every day.</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>She goes to class every day.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>correction</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Present Simple</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Beginner</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Choose the correct sentence.</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>I have a book.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Has / Have</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Beginner</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>I has a book.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>I have a book.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>I am have a book.</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>I having a book.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -524,142 +629,94 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Weekly Test Upload Template</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Use the Questions sheet for import. Do not rename the first-sheet headers.</t>
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Weekly Test Upload - Easy Guide</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Keep the first-row column names exactly the same.</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>question_text</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Required. Write the student-facing question.</t>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>1. question_text</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Required. Write the question students will see.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>expected_answer</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Strongly recommended for auto-checking and post-test answer key. Multiple valid answers: separate with ||</t>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>2. expected_answer</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Recommended. Used for automatic checking and the answer key.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>question_type</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Optional. Use: hindi_to_english, english_to_hindi, correction, short_answer, mcq</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>3. question_type</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Examples: hindi_to_english, english_to_hindi, correction, short_answer, mcq.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>topic_name</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Optional Admin metadata. It is not shown as a hint on the student paper/result.</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>4. option_a to option_d</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Fill only for MCQ. Leave blank for translation/correction/short answer.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>level</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Optional Admin metadata. Example: Beginner, Basic, Intermediate, Advanced.</t>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>5. Multiple accepted answers</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Separate valid answers with ||, for example: I cannot go || I can't go.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>marks</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Optional. Defaults to 1 if blank/invalid.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>option_a ... option_d</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Only required for MCQ. Leave blank for typed-answer questions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Example question</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>मुझे जाने दो।</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Example accepted answers</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Let me go. || Please let me go.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>No Excel file?</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Admin → Weekly Tests → Question Bank → Add one question manually. Manual entry and Excel upload save to the same question bank.</t>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Before upload</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>You may delete the 3 example rows and add your own questions. Do not rename the headers.</t>
         </is>
       </c>
     </row>

</xml_diff>